<commit_message>
Traitement automatique : Arbigny (retenter_erreurs/continuer)
</commit_message>
<xml_diff>
--- a/state/01016_arbigny.xlsx
+++ b/state/01016_arbigny.xlsx
@@ -12381,72 +12381,72 @@
       </c>
       <c r="ID3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ3" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR3" t="inlineStr">
@@ -29685,72 +29685,72 @@
       </c>
       <c r="ID10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ10" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR10" t="inlineStr">
@@ -32157,72 +32157,72 @@
       </c>
       <c r="ID11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ11" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR11" t="inlineStr">
@@ -34629,72 +34629,72 @@
       </c>
       <c r="ID12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ12" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR12" t="inlineStr">
@@ -37101,72 +37101,72 @@
       </c>
       <c r="ID13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ13" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR13" t="inlineStr">
@@ -39573,72 +39573,72 @@
       </c>
       <c r="ID14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ14" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR14" t="inlineStr">
@@ -42045,72 +42045,72 @@
       </c>
       <c r="ID15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ15" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR15" t="inlineStr">
@@ -44517,72 +44517,72 @@
       </c>
       <c r="ID16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ16" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR16" t="inlineStr">
@@ -46989,72 +46989,72 @@
       </c>
       <c r="ID17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ17" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR17" t="inlineStr">
@@ -49461,72 +49461,72 @@
       </c>
       <c r="ID18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ18" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR18" t="inlineStr">
@@ -51933,72 +51933,72 @@
       </c>
       <c r="ID19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IE19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IF19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IG19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IH19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="II19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IJ19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IK19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IL19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IM19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IN19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IO19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IP19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IQ19" t="inlineStr">
         <is>
-          <t>ERREUR</t>
+          <t>N</t>
         </is>
       </c>
       <c r="IR19" t="inlineStr">

</xml_diff>